<commit_message>
Updated negative test case and check for non-existent --CAT variable; Updated Description and Outcome.Message to make intention and error more clear.
</commit_message>
<xml_diff>
--- a/rules/CORE-000103/negative/01/data/unit-test-coreid-CG0429-negative.xlsx
+++ b/rules/CORE-000103/negative/01/data/unit-test-coreid-CG0429-negative.xlsx
@@ -9,6 +9,7 @@
     <sheet name="ag.xpt" sheetId="4" r:id="rId4"/>
     <sheet name="cm.xpt" sheetId="5" r:id="rId5"/>
     <sheet name="ex.xpt" sheetId="6" r:id="rId6"/>
+    <sheet name="mh.xpt" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -38,7 +39,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -64,14 +65,9 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -79,12 +75,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -120,7 +110,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -128,7 +118,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -626,7 +615,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -722,9 +711,49 @@
         <v>PRIOR DMARDS</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>mh.xpt</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>MHCAT</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>[ABSENT]</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>mh.xpt</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="2">
+        <v>5</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>MHSCAT</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>CARDIAC HISTORY</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -793,131 +822,131 @@
       <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Reported Agent Name</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Category for Agent</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Subcategory for Agent</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>AG Pre-Specified</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>AG Occurrence</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Dose per Administration</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="5" t="str">
         <v>Dose Description</v>
       </c>
-      <c r="L2" s="6" t="str">
+      <c r="L2" s="5" t="str">
         <v>Dose Units</v>
       </c>
-      <c r="M2" s="6" t="str">
+      <c r="M2" s="5" t="str">
         <v>Route of Administration</v>
       </c>
-      <c r="N2" s="6" t="str">
+      <c r="N2" s="5" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="O2" s="6" t="str">
+      <c r="O2" s="5" t="str">
         <v>End Date/Time of Agent</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="K3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="6" t="str">
+      <c r="K3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
-        <v>50</v>
-      </c>
-      <c r="B4" s="6">
-        <v>50</v>
-      </c>
-      <c r="C4" s="6">
-        <v>50</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="A4" s="5">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
-        <v>50</v>
-      </c>
-      <c r="F4" s="6">
-        <v>50</v>
-      </c>
-      <c r="G4" s="6">
-        <v>50</v>
-      </c>
-      <c r="H4" s="6">
-        <v>50</v>
-      </c>
-      <c r="I4" s="6">
-        <v>50</v>
-      </c>
-      <c r="J4" s="6">
-        <v>50</v>
-      </c>
-      <c r="K4" s="6">
-        <v>50</v>
-      </c>
-      <c r="L4" s="6">
-        <v>50</v>
-      </c>
-      <c r="M4" s="6">
-        <v>50</v>
-      </c>
-      <c r="N4" s="6">
-        <v>50</v>
-      </c>
-      <c r="O4" s="6">
+      <c r="E4" s="5">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5">
+        <v>50</v>
+      </c>
+      <c r="M4" s="5">
+        <v>50</v>
+      </c>
+      <c r="N4" s="5">
+        <v>50</v>
+      </c>
+      <c r="O4" s="5">
         <v>50</v>
       </c>
     </row>
@@ -937,10 +966,10 @@
       <c r="E5" s="4" t="str">
         <v>SALINE</v>
       </c>
-      <c r="F5" s="7" t="str">
+      <c r="F5" s="6" t="str">
         <v/>
       </c>
-      <c r="G5" s="7" t="str">
+      <c r="G5" s="6" t="str">
         <v>DFAJF</v>
       </c>
       <c r="H5" s="4" t="str">
@@ -1144,71 +1173,71 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Reported Name of Drug, Med, or Therapy</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Category for Medication</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Subcategory for Medication</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
-        <v>50</v>
-      </c>
-      <c r="B4" s="6">
-        <v>50</v>
-      </c>
-      <c r="C4" s="6">
-        <v>50</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="A4" s="5">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
-        <v>50</v>
-      </c>
-      <c r="F4" s="6">
-        <v>50</v>
-      </c>
-      <c r="G4" s="6">
+      <c r="E4" s="5">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5">
         <v>50</v>
       </c>
     </row>
@@ -1228,10 +1257,10 @@
       <c r="E5" s="4" t="str">
         <v>ASPIRIN</v>
       </c>
-      <c r="F5" s="7" t="str">
+      <c r="F5" s="6" t="str">
         <v/>
       </c>
-      <c r="G5" s="7" t="str">
+      <c r="G5" s="6" t="str">
         <v>PRIOR DMARDS</v>
       </c>
     </row>
@@ -1342,80 +1371,80 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Link ID</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Name of Treatment</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Category of Treatment</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Subcategory of Treatment</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
-        <v>50</v>
-      </c>
-      <c r="B4" s="6">
-        <v>50</v>
-      </c>
-      <c r="C4" s="6">
-        <v>50</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="A4" s="5">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
-        <v>50</v>
-      </c>
-      <c r="F4" s="6">
-        <v>50</v>
-      </c>
-      <c r="G4" s="6">
-        <v>50</v>
-      </c>
-      <c r="H4" s="6">
+      <c r="E4" s="5">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5">
         <v>50</v>
       </c>
     </row>
@@ -1499,4 +1528,115 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="str">
+        <v>STUDYID</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>DOMAIN</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>USUBJID</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>MHSEQ</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>MHTERM</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>MHSCAT</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="str">
+        <v>Study Identifier</v>
+      </c>
+      <c r="B2" s="5" t="str">
+        <v>Domain Abbreviation</v>
+      </c>
+      <c r="C2" s="5" t="str">
+        <v>Unique Subject Identifier</v>
+      </c>
+      <c r="D2" s="5" t="str">
+        <v>Sequence Number</v>
+      </c>
+      <c r="E2" s="5" t="str">
+        <v>Reported Medical History Term</v>
+      </c>
+      <c r="F2" s="5" t="str">
+        <v>Subcategory for Medical History</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5">
+        <v>8</v>
+      </c>
+      <c r="E4" s="5">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="str">
+        <v>XYZ</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <v>MH</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <v>XYZ-001-001</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <v>HYPERTENSION</v>
+      </c>
+      <c r="F5" s="6" t="str">
+        <v>CARDIAC HISTORY</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>